<commit_message>
Minor modifications to user help and manual
Clarify use of wet (bulk) density and dry density for model input parameters
</commit_message>
<xml_diff>
--- a/app/doc/Model parameters template.xlsx
+++ b/app/doc/Model parameters template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Matlab Code\MUImodels\muiApps\Asmita\doc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Matlab Code\muiModels\Asmita\app\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5864764F-2A60-4D38-A619-A028E138ECB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E6BEB38-BA0A-4E8B-8344-18D64580C737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3880" yWindow="2940" windowWidth="31540" windowHeight="16740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="97">
   <si>
     <t>concentration imported by advection (kg/m^3)</t>
   </si>
@@ -335,6 +335,15 @@
   </si>
   <si>
     <t>eq(4) in manual - method (i)</t>
+  </si>
+  <si>
+    <t>can be written</t>
+  </si>
+  <si>
+    <t>d=(pi/Tp)u((HA/ws)</t>
+  </si>
+  <si>
+    <t>di=(pi/Tp)^2 (tr/2)(V/ws)</t>
   </si>
 </sst>
 </file>
@@ -462,7 +471,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -708,6 +717,12 @@
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -733,9 +748,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -773,7 +788,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -879,7 +894,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1021,7 +1036,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1596,8 +1611,12 @@
       <c r="E25" s="76" t="s">
         <v>87</v>
       </c>
-      <c r="F25" s="76"/>
-      <c r="G25" s="76"/>
+      <c r="F25" s="95" t="s">
+        <v>94</v>
+      </c>
+      <c r="G25" s="76" t="s">
+        <v>95</v>
+      </c>
       <c r="H25" s="76"/>
       <c r="I25" s="76"/>
       <c r="J25" s="76"/>
@@ -1718,8 +1737,12 @@
       <c r="E30" s="77" t="s">
         <v>92</v>
       </c>
-      <c r="F30" s="77"/>
-      <c r="G30" s="77"/>
+      <c r="F30" s="94" t="s">
+        <v>94</v>
+      </c>
+      <c r="G30" s="77" t="s">
+        <v>96</v>
+      </c>
       <c r="H30" s="78"/>
       <c r="I30" s="78"/>
       <c r="J30" s="77"/>

</xml_diff>